<commit_message>
adding report and calibration_table
</commit_message>
<xml_diff>
--- a/outputs/match_sensors_output.xlsx
+++ b/outputs/match_sensors_output.xlsx
@@ -91,13 +91,13 @@
     <t>15:20:58</t>
   </si>
   <si>
-    <t>fixsensor-m2</t>
-  </si>
-  <si>
-    <t>fixsensor-m4</t>
-  </si>
-  <si>
-    <t>referenceiphone-m10</t>
+    <t>sensorA-m2</t>
+  </si>
+  <si>
+    <t>sensorA-m4</t>
+  </si>
+  <si>
+    <t>sensorB-m10</t>
   </si>
 </sst>
 </file>

</xml_diff>